<commit_message>
[Excel] Rename File & Remove Useless Colors
</commit_message>
<xml_diff>
--- a/tools/excel/netherlands/cbw_nis2.xlsx
+++ b/tools/excel/netherlands/cbw_nis2.xlsx
@@ -8,32 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JulianDoloir\Desktop\Repos\intuitem\ciso-assistant-community\tools\excel\netherlands\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F33459C-F8DB-4250-B528-7F827F9EA0A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F07A8965-2EB6-4648-90B0-709A8FEE7E4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5670" yWindow="-14400" windowWidth="19455" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1650" yWindow="-15870" windowWidth="25440" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
     <sheet name="fwk_meta" sheetId="2" r:id="rId2"/>
     <sheet name="fwk_content" sheetId="3" r:id="rId3"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">fwk_content!$A$1:$I$48</definedName>
-  </definedNames>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -79,6 +63,11 @@
     <t>description</t>
   </si>
   <si>
+    <t>## Introductie
+De evaluatietool is opgesteld als praktisch hulpmiddel om organisaties te ondersteunen bij het op een effectieve wijze verkrijgen van inzicht in de mate waarin zij voldoen aan de Cyberbeveiligingswet (Cbw) en het onderliggende Cyberbeveiligingsbesluit (Cbb).
+De evaluatietool is ontwikkeld om inzicht te geven in de huidige staat van cyberweerbaarheid en om verbeterpotentieel te identificeren, gebaseerd op de eisen zoals vastgelegd in de Cbw en Cbb. Het Cbw (NIS2) Control Framework vervangt de geldende wet- en regelgeving niet, maar maakt deze inzichtelijk en hanteerbaar - zie ook het studierapport vanaf p. 16. De Cbw en de Cbb dagen organisaties uit om middels risicoanalyse en inzicht in de eigen organisatie de Cbw en de Cbb te implementeren. Medewerkers van organisaties zijn zelf verantwoordelijk voor het kennen en naleven van de relevante wet- en regelgeving. Bovendien dient bij het gebruik ervan altijd rekening te worden gehouden met de specifieke context en kenmerken van de organisatie en haar omgeving.</t>
+  </si>
+  <si>
     <t>copyright</t>
   </si>
   <si>
@@ -103,6 +92,10 @@
   </si>
   <si>
     <t>description[en]</t>
+  </si>
+  <si>
+    <t>## Introduction
+The evaluation tool has been developed as a practical tool to support organizations in effectively gaining insight into their compliance with the Cybersecurity Act (Cbw) and the underlying Cybersecurity Decree (Cbb). The evaluation tool was developed to provide insight into the current state of cyber resilience and to identify potential for improvement, based on the requirements laid out in the Cbw and Cbb. The Cbw (NIS2) Control Framework does not replace current laws and regulations, but rather makes them transparent and manageable – see also the study report from p. 16 onwards. The Cbw and Cbb challenge organizations to implement the Cbw and Cbb through risk analysis and insight into their own organization. Employees of organizations are responsible for knowing and complying with the relevant laws and regulations. Furthermore, the specific context and characteristics of the organization and its environment should always be taken into account when using the tool.</t>
   </si>
   <si>
     <t>framework</t>
@@ -168,7 +161,17 @@
     <t>The entity has a security policy for its network and information systems, which includes (or refers to) appropriate and proportionate technical, organizational, and operational measures. This policy is actively applied, evaluated, and enforced (through a management system). The board establishes and periodically reviews the policy, and ensures that staff and other stakeholders are aware of it and act in accordance with it. This policy also defines the roles, responsibilities, and authorities related to the security of its network and information systems.</t>
   </si>
   <si>
-    <t>The measures shall include at least the following: a. policies on risk assessment and security of information systems; b. incident handling; c. business continuity, such as backup management and recovery plans, and crisis management; d. supply chain security, including security-related aspects of the relationships between the entity and its direct suppliers or service providers. e. security in the acquisition, development, and maintenance of network and information systems, including vulnerability response and disclosure; f. policies and procedures to assess the effectiveness of cybersecurity risk management measures; g. baseline cyber hygiene practices and cybersecurity training; h. policies and procedures on the use of cryptography and, where appropriate, encryption; i. security aspects related to personnel, access policies, and asset management; and j. where appropriate, the use of multi-factor authentication or continuous authentication solutions, secure voice, video, and text communications, and secure emergency communications systems within the entity.</t>
+    <t>The measures shall include at least the following:
+a. policies on risk assessment and security of information systems;
+b. incident handling;
+c. business continuity, such as backup management and recovery plans, and crisis management;
+d. supply chain security, including security-related aspects of the relationships between the entity and its direct suppliers or service providers.
+e. security in the acquisition, development, and maintenance of network and information systems, including vulnerability response and disclosure;
+f. policies and procedures to assess the effectiveness of cybersecurity risk management measures;
+g. baseline cyber hygiene practices and cybersecurity training;
+h. policies and procedures on the use of cryptography and, where appropriate, encryption;
+i. security aspects related to personnel, access policies, and asset management; and
+j. where appropriate, the use of multi-factor authentication or continuous authentication solutions, secure voice, video, and text communications, and secure emergency communications systems within the entity.</t>
   </si>
   <si>
     <t>Beleid over risicomanagement</t>
@@ -194,7 +197,11 @@
     <t>The entity has a risk management policy regarding the security of its network and information systems. This policy includes, at a minimum, a risk management methodology and risk acceptance criteria. Processes and procedures for risk analysis, risk assessment, and risk treatment are included for implementing the policy.Based on the risk analysis, the entity has an overview of the risks to its network and information systems. This overview is used to define security requirements for the network and information systems, and, if the risk analysis indicates the need, appropriate measures are taken.</t>
   </si>
   <si>
-    <t>When selecting measures, the entity must at least consider: - the state of the art; - the implementation costs; - where applicable, the relevant European and international standards; - the proportionality of the measures: the extent to which it is exposed to risks, the size of the entity, the likelihood of incidents occurring, and their severity (including their social and economic impact).</t>
+    <t>When selecting measures, the entity must at least consider:
+- the state of the art;
+- the implementation costs;
+- where applicable, the relevant European and international standards;
+- the proportionality of the measures: the extent to which it is exposed to risks, the size of the entity, the likelihood of incidents occurring, and their severity (including their social and economic impact).</t>
   </si>
   <si>
     <t>Evaluatie</t>
@@ -237,7 +244,13 @@
     <t>The entity has an incident management policy that is communicated and implemented. This policy defines the roles, responsibilities, and authorities regarding incident handling.</t>
   </si>
   <si>
-    <t>The policy establishes the roles, responsibilities, and authorities for: a. timely detection of incidents; b. analyzing and assessing incidents; c. responding to, mitigating the consequences of, eliminating the cause of, and recovering from incidents; d. documenting incidents; e. reporting incidents; and f. learning from incidents.</t>
+    <t>The policy establishes the roles, responsibilities, and authorities for:
+a. timely detection of incidents;
+b. analyzing and assessing incidents;
+c. responding to, mitigating the consequences of, eliminating the cause of, and recovering from incidents;
+d. documenting incidents;
+e. reporting incidents; and
+f. learning from incidents.</t>
   </si>
   <si>
     <t>4.2</t>
@@ -259,7 +272,13 @@
     <t>The entity has processes and procedures to monitor relevant activities, actions, and events in its network and information systems in order to detect, analyze, and classify incidents. The entity logs events relevant to the security of its network and information systems. The log files are stored for a predetermined period and protected from unauthorized modification.</t>
   </si>
   <si>
-    <t>These processes and procedures have been established and demonstrably applied, and include at least: a. timely detection of incidents; b. analysis and assessment of incidents; c. responding to, mitigating the consequences of, eliminating the cause of, and recovering from incidents; d. documenting incidents; e. reporting incidents; and f. learning from incidents.</t>
+    <t>These processes and procedures have been established and demonstrably applied, and include at least:
+a. timely detection of incidents;
+b. analysis and assessment of incidents;
+c. responding to, mitigating the consequences of, eliminating the cause of, and recovering from incidents;
+d. documenting incidents;
+e. reporting incidents; and
+f. learning from incidents.</t>
   </si>
   <si>
     <t>Bedrijfscontinuïteit en crisisbeheer</t>
@@ -308,7 +327,10 @@
     <t>The entity has a crisis management plan and tests and exercises this plan periodically.</t>
   </si>
   <si>
-    <t>The plan contains at least: a. the tasks, responsibilities and authorities for the staff in times of crisis, b.a description of the means of communication in times of crisis, c. where appropriate, a description of available emergency arrangements, including the use of secure emergency communications systems in times of crisis.</t>
+    <t>The plan contains at least:
+a. the tasks, responsibilities and authorities for the staff in times of crisis,
+b. a description of the means of communication in times of crisis,
+c. where appropriate, a description of available emergency arrangements, including the use of secure emergency communications systems in times of crisis.</t>
   </si>
   <si>
     <t>Beveiliging van de toeleveringsketen</t>
@@ -339,6 +361,12 @@
   </si>
   <si>
     <t>De entiteit heeft een volledige en actuele inventaris van haar leveranciers en dienstverleners en houdt deze bij. De entiteit houdt bij welke producten en diensten van leveranciers en dienstverleners worden afgenomen mede als de gemaakte afspreken over de afgenomen diensten en producten.</t>
+  </si>
+  <si>
+    <t>The entity has and maintains a complete and up-to-date inventory of its suppliers and service providers. The entity keeps track of which products and services are purchased from suppliers and service providers, also as well as the agreements made about the purchased services and products.</t>
+  </si>
+  <si>
+    <t>Notre: For "description[en]", Control 6.3 was missing in OG Framework (probably because the English version wasn't up to date (v1.1 available only, while NL version was at v1.2)). NL has been translated to English for this control</t>
   </si>
   <si>
     <t>Verwerven, ontwikkelen en onderhouden van informatiesystemen</t>
@@ -427,7 +455,11 @@
     <t>The entity has a policy on the use of cryptography and has established processes and procedures for the use of cryptography to implement this policy.</t>
   </si>
   <si>
-    <t>The policy shall at least specify: a. in which cases cryptography is used; b. in which cases, which types of encryption are used and how they are applied; c. who within the entity is responsible for implementing cryptography; d. who within the entity is responsible for key management.</t>
+    <t>The policy shall at least specify:
+a. in which cases cryptography is used;
+b. in which cases, which types of encryption are used and how they are applied;
+c. who within the entity is responsible for implementing cryptography;
+d. who within the entity is responsible for key management.</t>
   </si>
   <si>
     <t>Beveiligingsaspecten t.a.v. personeel</t>
@@ -483,7 +515,9 @@
     <t>The entity has a policy for the management of its assets used in the conduct of its operations or in the provision of its services and has asset management processes and procedures to implement that policy.</t>
   </si>
   <si>
-    <t>The policy should include at least: a. a system for classifying assets at different levels, where applicable, based on confidentiality, integrity, and availability requirements; b. rules for the acceptable use of assets.</t>
+    <t>The policy should include at least:
+a. a system for classifying assets at different levels, where applicable, based on confidentiality, integrity, and availability requirements;
+b. rules for the acceptable use of assets.</t>
   </si>
   <si>
     <t>12.2</t>
@@ -550,7 +584,17 @@
     <t>Following training, the entity's board is able to identify security risks to network and information systems and assess their impact on the services provided by the entity. Furthermore, the training ensures that each board member is able to assess cybersecurity risk management measures and their impact on the services provided by the entity.</t>
   </si>
   <si>
-    <t>The training shall, at a minimum, cover the following topics: a. The types of risks for network and information systems; b. Risk management processes; c. Risk assessment methodology; d. Cybersecurity risk control measures (as also laid down in security policy). The training certificate shall, at a minimum, include: a. The name of the board member of the entity; b. The date(s) on which the training was completed; c. The topics covered in the training; and d. The name of the training provider. The training certificate shall be available in Dutch or English.</t>
+    <t>The training shall, at a minimum, cover the following topics:
+a. The types of risks for network and information systems;
+b. Risk management processes;
+c. Risk assessment methodology;
+d. Cybersecurity risk control measures (as also laid down in security policy).
+The training certificate shall, at a minimum, include:
+a. The name of the board member of the entity;
+b. The date(s) on which the training was completed;
+c. The topics covered in the training; and
+d. The name of the training provider.
+The training certificate shall be available in Dutch or English.</t>
   </si>
   <si>
     <t>14.2</t>
@@ -589,7 +633,10 @@
     <t>The entity shall report any significant incident to its CSIRT and the competent authority.</t>
   </si>
   <si>
-    <t>An incident is significant if it: a. causes or may cause serious operational disruption of services or financial loss to the entity concerned; or b. has affected or may affect other entities by causing significant material or immaterial damage. Voluntary reporting obligation: Every entity has the option to voluntarily report an incident, near miss, or cyber threat to its CSIRT or competent authority.</t>
+    <t>An incident is significant if it:
+a. causes or may cause serious operational disruption of services or financial loss to the entity concerned; or
+b. has affected or may affect other entities by causing significant material or immaterial damage.
+Voluntary reporting obligation: Every entity has the option to voluntarily report an incident, near miss, or cyber threat to its CSIRT or competent authority.</t>
   </si>
   <si>
     <t>Vroegtijdige waarschuwing</t>
@@ -615,7 +662,22 @@
     <t>The entity reports significant incidents in three phases: 1) the initial (early) notification is made without delay or, if that is not possible, within 24 hours of becoming aware of the significant incident. 2) an interim update on the incident's development (within 72 hours of submitting the initial notification, even if the status or handling of the incident has not changed or if regular activities have resumed); and 3) the final report with a root cause analysis and follow-up actions (no later than one month after submitting the interim update). If the incident is still ongoing at the time of this report, this report becomes an interim report. In this case, the final report follows within one month of the incident's resolution.</t>
   </si>
   <si>
-    <t>In the early notification, the entity shall provide the following information: a. an indication of whether the incident is likely to have been caused by an unlawful or malicious act; b. whether the incident may have cross-border implications; c. the contact details of the official responsible for notification; d. the estimated time of onset of the significant incident,e. where possible; a description of the nature and currently noticeable impact of the incident, f. where possible; a forecast of the recovery time; and, g. where possible, the measures taken or planned by the entity to mitigate the impact of the significant incident or prevent its recurrence. In the interim update, the entity shall provide a. an update on the information from the early notification and, b. where applicable, an initial assessment of the significant incident, including its severity and impact, the indicators of impairment, and any available information enabling the CSIRT and the competent authority to determine any cross-border implications of the incident. The final report shall include a. a detailed description of the incident, its severity and consequences, b. the type of threat or root cause likely to have led to the incident, c. risk mitigation measures implemented and ongoing, and, d. where appropriate, the transboundary implications of the incident.</t>
+    <t>In the early notification, the entity shall provide the following information:
+a. an indication of whether the incident is likely to have been caused by an unlawful or malicious act;
+b. whether the incident may have cross-border implications;
+c. the contact details of the official responsible for notification;
+d. the estimated time of onset of the significant incident,
+e. where possible; a description of the nature and currently noticeable impact of the incident,
+f. where possible; a forecast of the recovery time; and,
+g. where possible, the measures taken or planned by the entity to mitigate the impact of the significant incident or prevent its recurrence.
+In the interim update, the entity shall provide
+a. an update on the information from the early notification and,
+b. where applicable, an initial assessment of the significant incident, including its severity and impact, the indicators of impairment, and any available information enabling the CSIRT and the competent authority to determine any cross-border implications of the incident.
+The final report shall include
+a. a detailed description of the incident, its severity and consequences,
+b. the type of threat or root cause likely to have led to the incident,
+c. risk mitigation measures implemented and ongoing, and,
+d. where appropriate, the transboundary implications of the incident.</t>
   </si>
   <si>
     <t>Nadere regels over meldingen</t>
@@ -631,21 +693,6 @@
   </si>
   <si>
     <t>In the event of a significant incident, the entity will notify the recipients of its services as soon as possible if the incident could adversely affect service provision. The entity will also communicate the measures these recipients can take in response to the threat.</t>
-  </si>
-  <si>
-    <t>The entity has and maintains a complete and up-to-date inventory of its suppliers and service providers. The entity keeps track of which products and services are purchased from suppliers and service providers, also as well as the agreements made about the purchased services and products.</t>
-  </si>
-  <si>
-    <t>Notre: For "description[en]", Control 6.3 was missing in OG Framework (probably because the English version wasn't up to date (v1.1 available only, while NL version was at v1.2)). NL has been translated to English for this control</t>
-  </si>
-  <si>
-    <t>## Introductie
-De evaluatietool is opgesteld als praktisch hulpmiddel om organisaties te ondersteunen bij het op een effectieve wijze verkrijgen van inzicht in de mate waarin zij voldoen aan de Cyberbeveiligingswet (Cbw) en het onderliggende Cyberbeveiligingsbesluit (Cbb).
-De evaluatietool is ontwikkeld om inzicht te geven in de huidige staat van cyberweerbaarheid en om verbeterpotentieel te identificeren, gebaseerd op de eisen zoals vastgelegd in de Cbw en Cbb. Het Cbw (NIS2) Control Framework vervangt de geldende wet- en regelgeving niet, maar maakt deze inzichtelijk en hanteerbaar - zie ook het studierapport vanaf p. 16. De Cbw en de Cbb dagen organisaties uit om middels risicoanalyse en inzicht in de eigen organisatie de Cbw en de Cbb te implementeren. Medewerkers van organisaties zijn zelf verantwoordelijk voor het kennen en naleven van de relevante wet- en regelgeving. Bovendien dient bij het gebruik ervan altijd rekening te worden gehouden met de specifieke context en kenmerken van de organisatie en haar omgeving.</t>
-  </si>
-  <si>
-    <t>## Introduction
-The evaluation tool has been developed as a practical tool to support organizations in effectively gaining insight into their compliance with the Cybersecurity Act (Cbw) and the underlying Cybersecurity Decree (Cbb). The evaluation tool was developed to provide insight into the current state of cyber resilience and to identify potential for improvement, based on the requirements laid out in the Cbw and Cbb. The Cbw (NIS2) Control Framework does not replace current laws and regulations, but rather makes them transparent and manageable – see also the study report from p. 16 onwards. The Cbw and Cbb challenge organizations to implement the Cbw and Cbb through risk analysis and insight into their own organization. Employees of organizations are responsible for knowing and complying with the relevant laws and regulations. Furthermore, the specific context and characteristics of the organization and its environment should always be taken into account when using the tool.</t>
   </si>
 </sst>
 </file>
@@ -701,7 +748,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -716,43 +763,46 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="11">
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -768,18 +818,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FAA93575-958B-48B3-8547-389756FF2907}" name="Tableau1" displayName="Tableau1" ref="A1:I48" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
-  <autoFilter ref="A1:I48" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tableau1" displayName="Tableau1" ref="A1:I48" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+  <autoFilter ref="A1:I48" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{AE25FFF5-D7E2-4BA8-86E6-E9516C7A9EC9}" name="assessable" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{E8C41B82-7285-445D-8BEA-4E8A7DEF6B5F}" name="depth" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{A5ACFCD9-3394-4958-8ABE-148DA23E5812}" name="ref_id" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{C7FEDC4E-CA1A-418C-8A2B-E46BB864E30D}" name="name" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{C66C759A-558C-4DFF-8494-FB85DBFBBD57}" name="description" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{5F1BAD77-792F-4658-A23E-678D7BBCDAC1}" name="annotation" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{5603FCE9-8084-4EE9-B623-4050A8947988}" name="name[en]" dataDxfId="2"/>
-    <tableColumn id="9" xr3:uid="{F41AAF1E-63A7-4C35-8EE6-10FB1539CB14}" name="description[en]" dataDxfId="1"/>
-    <tableColumn id="10" xr3:uid="{30A571C8-7147-4849-BF08-4AF6393D258F}" name="annotation[en]" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="assessable" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="depth" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="ref_id" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="name" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="description" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="annotation" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="name[en]" dataDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="description[en]" dataDxfId="1"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="annotation[en]" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1125,52 +1175,52 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="201.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" ht="201.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="72" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="172.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" ht="172.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>179</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -1192,15 +1242,15 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -1208,7 +1258,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -1227,28 +1277,28 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="201.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" ht="201.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>178</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="172.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" ht="172.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>179</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -1272,10 +1322,10 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>8</v>
@@ -1287,16 +1337,16 @@
         <v>12</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
@@ -1306,12 +1356,12 @@
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
@@ -1323,39 +1373,39 @@
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
     </row>
-    <row r="4" spans="1:9" ht="259.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="259.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B4" s="1">
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -1365,39 +1415,39 @@
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
       <c r="G5" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
     </row>
-    <row r="6" spans="1:9" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B6" s="1">
         <v>3</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -1407,34 +1457,34 @@
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
       <c r="G7" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
     </row>
-    <row r="8" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B8" s="1">
         <v>3</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I8" s="1"/>
     </row>
@@ -1445,64 +1495,64 @@
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
     </row>
-    <row r="10" spans="1:9" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B10" s="1">
         <v>3</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G10" s="1"/>
       <c r="H10" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="144" x14ac:dyDescent="0.3">
+        <v>58</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="144" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B11" s="1">
         <v>3</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="G11" s="1"/>
       <c r="H11" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
@@ -1512,85 +1562,85 @@
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
       <c r="G12" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
     </row>
-    <row r="13" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B13" s="1">
         <v>3</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G13" s="1"/>
       <c r="H13" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B14" s="1">
         <v>3</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I14" s="1"/>
     </row>
-    <row r="15" spans="1:9" ht="72" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B15" s="1">
         <v>3</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G15" s="1"/>
       <c r="H15" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
@@ -1600,80 +1650,80 @@
       </c>
       <c r="C16" s="1"/>
       <c r="D16" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
       <c r="G16" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
     </row>
-    <row r="17" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B17" s="1">
         <v>3</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D17" s="1"/>
       <c r="E17" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I17" s="1"/>
     </row>
-    <row r="18" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B18" s="1">
         <v>3</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D18" s="1"/>
       <c r="E18" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="I18" s="1"/>
     </row>
-    <row r="19" spans="1:10" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" ht="62.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B19" s="1">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D19" s="1"/>
       <c r="E19" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="3" t="s">
-        <v>176</v>
+        <v>90</v>
       </c>
       <c r="I19" s="1"/>
       <c r="J19" s="4" t="s">
-        <v>177</v>
+        <v>91</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
@@ -1683,80 +1733,80 @@
       </c>
       <c r="C20" s="1"/>
       <c r="D20" s="1" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
       <c r="G20" s="1" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
     </row>
-    <row r="21" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B21" s="1">
         <v>3</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="D21" s="1"/>
       <c r="E21" s="1" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="G21" s="1"/>
       <c r="H21" s="1" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B22" s="1">
         <v>3</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I22" s="1"/>
     </row>
-    <row r="23" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B23" s="1">
         <v>3</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I23" s="1"/>
     </row>
@@ -1767,55 +1817,55 @@
       </c>
       <c r="C24" s="1"/>
       <c r="D24" s="1" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
       <c r="G24" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
     </row>
-    <row r="25" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B25" s="1">
         <v>3</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
       <c r="H25" s="1" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="I25" s="1"/>
     </row>
-    <row r="26" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B26" s="1">
         <v>3</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="D26" s="1"/>
       <c r="E26" s="1" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
       <c r="H26" s="1" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="I26" s="1"/>
     </row>
@@ -1826,39 +1876,39 @@
       </c>
       <c r="C27" s="1"/>
       <c r="D27" s="1" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
       <c r="G27" s="1" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
     </row>
-    <row r="28" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B28" s="1">
         <v>3</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D28" s="1"/>
       <c r="E28" s="1" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="G28" s="1"/>
       <c r="H28" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>115</v>
+        <v>118</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
@@ -1868,34 +1918,34 @@
       </c>
       <c r="C29" s="1"/>
       <c r="D29" s="1" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
       <c r="G29" s="1" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
     </row>
-    <row r="30" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B30" s="1">
         <v>3</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D30" s="1"/>
       <c r="E30" s="1" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
       <c r="H30" s="1" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="I30" s="1"/>
     </row>
@@ -1906,34 +1956,34 @@
       </c>
       <c r="C31" s="1"/>
       <c r="D31" s="1" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
       <c r="G31" s="1" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
     </row>
-    <row r="32" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B32" s="1">
         <v>3</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="D32" s="1"/>
       <c r="E32" s="1" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
       <c r="H32" s="1" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="I32" s="1"/>
     </row>
@@ -1944,59 +1994,59 @@
       </c>
       <c r="C33" s="1"/>
       <c r="D33" s="1" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
       <c r="G33" s="1" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
     </row>
-    <row r="34" spans="1:9" ht="72" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B34" s="1">
         <v>3</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="D34" s="1"/>
       <c r="E34" s="1" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="G34" s="1"/>
       <c r="H34" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="I34" s="1" t="s">
-        <v>132</v>
+        <v>135</v>
+      </c>
+      <c r="I34" s="5" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B35" s="1">
         <v>3</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D35" s="1"/>
       <c r="E35" s="1" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="F35" s="1"/>
       <c r="G35" s="1"/>
       <c r="H35" s="1" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="I35" s="1"/>
     </row>
@@ -2007,39 +2057,39 @@
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
       <c r="G36" s="1" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="H36" s="1"/>
       <c r="I36" s="1"/>
     </row>
-    <row r="37" spans="1:9" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B37" s="1">
         <v>3</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D37" s="1"/>
       <c r="E37" s="1" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="G37" s="1"/>
       <c r="H37" s="1" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
@@ -2049,12 +2099,12 @@
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
       <c r="G38" s="1" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
@@ -2066,59 +2116,59 @@
       </c>
       <c r="C39" s="1"/>
       <c r="D39" s="1" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
       <c r="G39" s="1" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="H39" s="1"/>
       <c r="I39" s="1"/>
     </row>
-    <row r="40" spans="1:9" ht="172.8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" ht="172.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B40" s="1">
         <v>3</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D40" s="1"/>
       <c r="E40" s="1" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="G40" s="1"/>
       <c r="H40" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="I40" s="1" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+        <v>154</v>
+      </c>
+      <c r="I40" s="5" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B41" s="1">
         <v>3</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D41" s="1"/>
       <c r="E41" s="1" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="F41" s="1"/>
       <c r="G41" s="1"/>
       <c r="H41" s="1" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="I41" s="1"/>
     </row>
@@ -2129,12 +2179,12 @@
       </c>
       <c r="C42" s="1"/>
       <c r="D42" s="1" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
       <c r="G42" s="1" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="H42" s="1"/>
       <c r="I42" s="1"/>
@@ -2146,39 +2196,39 @@
       </c>
       <c r="C43" s="1"/>
       <c r="D43" s="1" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
       <c r="G43" s="1" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="H43" s="1"/>
       <c r="I43" s="1"/>
     </row>
-    <row r="44" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B44" s="1">
         <v>3</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="D44" s="1"/>
       <c r="E44" s="1" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="G44" s="1"/>
       <c r="H44" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="I44" s="1" t="s">
-        <v>163</v>
+        <v>166</v>
+      </c>
+      <c r="I44" s="5" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.3">
@@ -2188,39 +2238,39 @@
       </c>
       <c r="C45" s="1"/>
       <c r="D45" s="1" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
       <c r="G45" s="1" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="H45" s="1"/>
       <c r="I45" s="1"/>
     </row>
-    <row r="46" spans="1:9" ht="259.2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" ht="259.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B46" s="1">
         <v>3</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="D46" s="1"/>
       <c r="E46" s="1" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="G46" s="1"/>
       <c r="H46" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="I46" s="1" t="s">
-        <v>170</v>
+        <v>173</v>
+      </c>
+      <c r="I46" s="5" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.3">
@@ -2230,34 +2280,34 @@
       </c>
       <c r="C47" s="1"/>
       <c r="D47" s="1" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
       <c r="G47" s="1" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="H47" s="1"/>
       <c r="I47" s="1"/>
     </row>
-    <row r="48" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B48" s="1">
         <v>3</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="D48" s="1"/>
       <c r="E48" s="1" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F48" s="1"/>
       <c r="G48" s="1"/>
       <c r="H48" s="1" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="I48" s="1"/>
     </row>

</xml_diff>

<commit_message>
[Excel] Add Missing 14.2 Annotation (NL & EN)
</commit_message>
<xml_diff>
--- a/tools/excel/netherlands/cbw_nis2.xlsx
+++ b/tools/excel/netherlands/cbw_nis2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JulianDoloir\Desktop\Repos\intuitem\ciso-assistant-community\tools\excel\netherlands\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F07A8965-2EB6-4648-90B0-709A8FEE7E4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA8B3A55-9824-4B2C-A790-B7431564389E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1650" yWindow="-15870" windowWidth="25440" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1764" yWindow="684" windowWidth="19452" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="180">
   <si>
     <t>type</t>
   </si>
@@ -748,7 +748,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -762,9 +762,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1383,7 +1380,7 @@
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
     </row>
-    <row r="4" spans="1:9" ht="259.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>35</v>
       </c>
@@ -1404,7 +1401,7 @@
       <c r="H4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" s="1" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1425,7 +1422,7 @@
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
     </row>
-    <row r="6" spans="1:9" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>35</v>
       </c>
@@ -1446,7 +1443,7 @@
       <c r="H6" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="I6" s="1" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1467,7 +1464,7 @@
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
     </row>
-    <row r="8" spans="1:9" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>35</v>
       </c>
@@ -1505,7 +1502,7 @@
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
     </row>
-    <row r="10" spans="1:9" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>35</v>
       </c>
@@ -1526,11 +1523,11 @@
       <c r="H10" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="I10" s="1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="144" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="144" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>35</v>
       </c>
@@ -1551,7 +1548,7 @@
       <c r="H11" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="I11" s="1" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1572,7 +1569,7 @@
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
     </row>
-    <row r="13" spans="1:9" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>35</v>
       </c>
@@ -1597,7 +1594,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>35</v>
       </c>
@@ -1618,7 +1615,7 @@
       </c>
       <c r="I14" s="1"/>
     </row>
-    <row r="15" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="72" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>35</v>
       </c>
@@ -1639,7 +1636,7 @@
       <c r="H15" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="I15" s="5" t="s">
+      <c r="I15" s="1" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1660,7 +1657,7 @@
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
     </row>
-    <row r="17" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>35</v>
       </c>
@@ -1681,7 +1678,7 @@
       </c>
       <c r="I17" s="1"/>
     </row>
-    <row r="18" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>35</v>
       </c>
@@ -1702,7 +1699,7 @@
       </c>
       <c r="I18" s="1"/>
     </row>
-    <row r="19" spans="1:10" ht="62.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>35</v>
       </c>
@@ -1743,7 +1740,7 @@
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
     </row>
-    <row r="21" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>35</v>
       </c>
@@ -1768,7 +1765,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>35</v>
       </c>
@@ -1789,7 +1786,7 @@
       </c>
       <c r="I22" s="1"/>
     </row>
-    <row r="23" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>35</v>
       </c>
@@ -1827,7 +1824,7 @@
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
     </row>
-    <row r="25" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>35</v>
       </c>
@@ -1848,7 +1845,7 @@
       </c>
       <c r="I25" s="1"/>
     </row>
-    <row r="26" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>35</v>
       </c>
@@ -1886,7 +1883,7 @@
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
     </row>
-    <row r="28" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>35</v>
       </c>
@@ -1907,7 +1904,7 @@
       <c r="H28" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="I28" s="5" t="s">
+      <c r="I28" s="1" t="s">
         <v>119</v>
       </c>
     </row>
@@ -1928,7 +1925,7 @@
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
     </row>
-    <row r="30" spans="1:10" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>35</v>
       </c>
@@ -1966,7 +1963,7 @@
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
     </row>
-    <row r="32" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>35</v>
       </c>
@@ -2004,7 +2001,7 @@
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
     </row>
-    <row r="34" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" ht="72" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>35</v>
       </c>
@@ -2025,7 +2022,7 @@
       <c r="H34" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="I34" s="5" t="s">
+      <c r="I34" s="1" t="s">
         <v>136</v>
       </c>
     </row>
@@ -2067,7 +2064,7 @@
       <c r="H36" s="1"/>
       <c r="I36" s="1"/>
     </row>
-    <row r="37" spans="1:9" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>35</v>
       </c>
@@ -2126,7 +2123,7 @@
       <c r="H39" s="1"/>
       <c r="I39" s="1"/>
     </row>
-    <row r="40" spans="1:9" ht="172.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>35</v>
       </c>
@@ -2147,11 +2144,11 @@
       <c r="H40" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="I40" s="5" t="s">
+      <c r="I40" s="1" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>35</v>
       </c>
@@ -2165,12 +2162,16 @@
       <c r="E41" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="F41" s="1"/>
+      <c r="F41" s="1" t="s">
+        <v>153</v>
+      </c>
       <c r="G41" s="1"/>
       <c r="H41" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="I41" s="1"/>
+      <c r="I41" s="1" t="s">
+        <v>155</v>
+      </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
@@ -2206,7 +2207,7 @@
       <c r="H43" s="1"/>
       <c r="I43" s="1"/>
     </row>
-    <row r="44" spans="1:9" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>35</v>
       </c>
@@ -2227,7 +2228,7 @@
       <c r="H44" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="I44" s="5" t="s">
+      <c r="I44" s="1" t="s">
         <v>167</v>
       </c>
     </row>
@@ -2248,7 +2249,7 @@
       <c r="H45" s="1"/>
       <c r="I45" s="1"/>
     </row>
-    <row r="46" spans="1:9" ht="259.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>35</v>
       </c>
@@ -2269,7 +2270,7 @@
       <c r="H46" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="I46" s="5" t="s">
+      <c r="I46" s="1" t="s">
         <v>174</v>
       </c>
     </row>
@@ -2290,7 +2291,7 @@
       <c r="H47" s="1"/>
       <c r="I47" s="1"/>
     </row>
-    <row r="48" spans="1:9" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>35</v>
       </c>

</xml_diff>

<commit_message>
Fix "description[en]" Text Formatting in "library_meta" & "fwk_meta"
</commit_message>
<xml_diff>
--- a/tools/excel/netherlands/cbw_nis2.xlsx
+++ b/tools/excel/netherlands/cbw_nis2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JulianDoloir\Desktop\Repos\intuitem\ciso-assistant-community\tools\excel\netherlands\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA8B3A55-9824-4B2C-A790-B7431564389E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{782F7146-0AB4-4BA4-9DD2-943959E07E29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1764" yWindow="684" windowWidth="19452" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
@@ -92,10 +92,6 @@
   </si>
   <si>
     <t>description[en]</t>
-  </si>
-  <si>
-    <t>## Introduction
-The evaluation tool has been developed as a practical tool to support organizations in effectively gaining insight into their compliance with the Cybersecurity Act (Cbw) and the underlying Cybersecurity Decree (Cbb). The evaluation tool was developed to provide insight into the current state of cyber resilience and to identify potential for improvement, based on the requirements laid out in the Cbw and Cbb. The Cbw (NIS2) Control Framework does not replace current laws and regulations, but rather makes them transparent and manageable – see also the study report from p. 16 onwards. The Cbw and Cbb challenge organizations to implement the Cbw and Cbb through risk analysis and insight into their own organization. Employees of organizations are responsible for knowing and complying with the relevant laws and regulations. Furthermore, the specific context and characteristics of the organization and its environment should always be taken into account when using the tool.</t>
   </si>
   <si>
     <t>framework</t>
@@ -693,6 +689,11 @@
   </si>
   <si>
     <t>In the event of a significant incident, the entity will notify the recipients of its services as soon as possible if the incident could adversely affect service provision. The entity will also communicate the measures these recipients can take in response to the threat.</t>
+  </si>
+  <si>
+    <t>## Introduction
+The evaluation tool has been developed as a practical tool to support organizations in effectively gaining insight into their compliance with the Cybersecurity Act (Cbw) and the underlying Cybersecurity Decree (Cbb).
+The evaluation tool was developed to provide insight into the current state of cyber resilience and to identify potential for improvement, based on the requirements laid out in the Cbw and Cbb. The Cbw (NIS2) Control Framework does not replace current laws and regulations, but rather makes them transparent and manageable – see also the study report from p. 16 onwards. The Cbw and Cbb challenge organizations to implement the Cbw and Cbb through risk analysis and insight into their own organization. Employees of organizations are responsible for knowing and complying with the relevant laws and regulations. Furthermore, the specific context and characteristics of the organization and its environment should always be taken into account when using the tool.</t>
   </si>
 </sst>
 </file>
@@ -1212,12 +1213,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="172.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>22</v>
+        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -1239,15 +1240,15 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -1255,7 +1256,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -1294,8 +1295,8 @@
       <c r="A8" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>22</v>
+      <c r="B8" s="2" t="s">
+        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -1319,10 +1320,10 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>28</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>8</v>
@@ -1334,7 +1335,7 @@
         <v>12</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>20</v>
@@ -1343,7 +1344,7 @@
         <v>21</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
@@ -1353,12 +1354,12 @@
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
@@ -1370,39 +1371,39 @@
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
     </row>
     <row r="4" spans="1:9" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" s="1">
+        <v>3</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="B4" s="1">
-        <v>3</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>38</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -1412,39 +1413,39 @@
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
       <c r="G5" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
     </row>
     <row r="6" spans="1:9" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B6" s="1">
         <v>3</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>45</v>
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I6" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -1454,34 +1455,34 @@
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
       <c r="G7" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
     </row>
     <row r="8" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B8" s="1">
         <v>3</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I8" s="1"/>
     </row>
@@ -1492,64 +1493,64 @@
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
     </row>
     <row r="10" spans="1:9" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B10" s="1">
         <v>3</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>57</v>
       </c>
       <c r="G10" s="1"/>
       <c r="H10" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="I10" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="144" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B11" s="1">
         <v>3</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>62</v>
       </c>
       <c r="G11" s="1"/>
       <c r="H11" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="I11" s="1" t="s">
         <v>63</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
@@ -1559,85 +1560,85 @@
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
       <c r="G12" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
     </row>
     <row r="13" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B13" s="1">
         <v>3</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>69</v>
       </c>
       <c r="G13" s="1"/>
       <c r="H13" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="I13" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B14" s="1">
         <v>3</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I14" s="1"/>
     </row>
     <row r="15" spans="1:9" ht="72" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B15" s="1">
         <v>3</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>76</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>77</v>
       </c>
       <c r="G15" s="1"/>
       <c r="H15" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="I15" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
@@ -1647,80 +1648,80 @@
       </c>
       <c r="C16" s="1"/>
       <c r="D16" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
       <c r="G16" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
     </row>
     <row r="17" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B17" s="1">
         <v>3</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D17" s="1"/>
       <c r="E17" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I17" s="1"/>
     </row>
     <row r="18" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B18" s="1">
         <v>3</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D18" s="1"/>
       <c r="E18" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I18" s="1"/>
     </row>
     <row r="19" spans="1:10" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B19" s="1">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D19" s="1"/>
       <c r="E19" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I19" s="1"/>
       <c r="J19" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
@@ -1730,80 +1731,80 @@
       </c>
       <c r="C20" s="1"/>
       <c r="D20" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
       <c r="G20" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
     </row>
     <row r="21" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B21" s="1">
         <v>3</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D21" s="1"/>
       <c r="E21" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>95</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>96</v>
       </c>
       <c r="G21" s="1"/>
       <c r="H21" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="I21" s="1" t="s">
         <v>97</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B22" s="1">
         <v>3</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I22" s="1"/>
     </row>
     <row r="23" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B23" s="1">
         <v>3</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I23" s="1"/>
     </row>
@@ -1814,55 +1815,55 @@
       </c>
       <c r="C24" s="1"/>
       <c r="D24" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
       <c r="G24" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
     </row>
     <row r="25" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B25" s="1">
         <v>3</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
       <c r="H25" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I25" s="1"/>
     </row>
     <row r="26" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B26" s="1">
         <v>3</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D26" s="1"/>
       <c r="E26" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
       <c r="H26" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I26" s="1"/>
     </row>
@@ -1873,39 +1874,39 @@
       </c>
       <c r="C27" s="1"/>
       <c r="D27" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
       <c r="G27" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
     </row>
     <row r="28" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B28" s="1">
         <v>3</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D28" s="1"/>
       <c r="E28" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F28" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>117</v>
       </c>
       <c r="G28" s="1"/>
       <c r="H28" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="I28" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
@@ -1915,34 +1916,34 @@
       </c>
       <c r="C29" s="1"/>
       <c r="D29" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
       <c r="G29" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
     </row>
     <row r="30" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B30" s="1">
         <v>3</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D30" s="1"/>
       <c r="E30" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
       <c r="H30" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I30" s="1"/>
     </row>
@@ -1953,34 +1954,34 @@
       </c>
       <c r="C31" s="1"/>
       <c r="D31" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
       <c r="G31" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
     </row>
     <row r="32" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B32" s="1">
         <v>3</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D32" s="1"/>
       <c r="E32" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
       <c r="H32" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I32" s="1"/>
     </row>
@@ -1991,59 +1992,59 @@
       </c>
       <c r="C33" s="1"/>
       <c r="D33" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
       <c r="G33" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
     </row>
     <row r="34" spans="1:9" ht="72" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B34" s="1">
         <v>3</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D34" s="1"/>
       <c r="E34" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="F34" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>134</v>
       </c>
       <c r="G34" s="1"/>
       <c r="H34" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="I34" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="I34" s="1" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B35" s="1">
         <v>3</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D35" s="1"/>
       <c r="E35" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F35" s="1"/>
       <c r="G35" s="1"/>
       <c r="H35" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I35" s="1"/>
     </row>
@@ -2054,39 +2055,39 @@
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
       <c r="G36" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H36" s="1"/>
       <c r="I36" s="1"/>
     </row>
     <row r="37" spans="1:9" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B37" s="1">
         <v>3</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D37" s="1"/>
       <c r="E37" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F37" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>144</v>
       </c>
       <c r="G37" s="1"/>
       <c r="H37" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="I37" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="I37" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
@@ -2096,12 +2097,12 @@
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
       <c r="G38" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
@@ -2113,64 +2114,64 @@
       </c>
       <c r="C39" s="1"/>
       <c r="D39" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
       <c r="G39" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H39" s="1"/>
       <c r="I39" s="1"/>
     </row>
     <row r="40" spans="1:9" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B40" s="1">
         <v>3</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D40" s="1"/>
       <c r="E40" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="F40" s="1" t="s">
         <v>152</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>153</v>
       </c>
       <c r="G40" s="1"/>
       <c r="H40" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="I40" s="1" t="s">
         <v>154</v>
-      </c>
-      <c r="I40" s="1" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="41" spans="1:9" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B41" s="1">
         <v>3</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D41" s="1"/>
       <c r="E41" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G41" s="1"/>
       <c r="H41" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
@@ -2180,12 +2181,12 @@
       </c>
       <c r="C42" s="1"/>
       <c r="D42" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
       <c r="G42" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="H42" s="1"/>
       <c r="I42" s="1"/>
@@ -2197,39 +2198,39 @@
       </c>
       <c r="C43" s="1"/>
       <c r="D43" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
       <c r="G43" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H43" s="1"/>
       <c r="I43" s="1"/>
     </row>
     <row r="44" spans="1:9" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B44" s="1">
         <v>3</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D44" s="1"/>
       <c r="E44" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="F44" s="1" t="s">
         <v>164</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>165</v>
       </c>
       <c r="G44" s="1"/>
       <c r="H44" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="I44" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="I44" s="1" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.3">
@@ -2239,39 +2240,39 @@
       </c>
       <c r="C45" s="1"/>
       <c r="D45" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
       <c r="G45" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H45" s="1"/>
       <c r="I45" s="1"/>
     </row>
     <row r="46" spans="1:9" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B46" s="1">
         <v>3</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D46" s="1"/>
       <c r="E46" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="F46" s="1" t="s">
         <v>171</v>
-      </c>
-      <c r="F46" s="1" t="s">
-        <v>172</v>
       </c>
       <c r="G46" s="1"/>
       <c r="H46" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="I46" s="1" t="s">
         <v>173</v>
-      </c>
-      <c r="I46" s="1" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.3">
@@ -2281,34 +2282,34 @@
       </c>
       <c r="C47" s="1"/>
       <c r="D47" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
       <c r="G47" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="H47" s="1"/>
       <c r="I47" s="1"/>
     </row>
     <row r="48" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B48" s="1">
         <v>3</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D48" s="1"/>
       <c r="E48" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F48" s="1"/>
       <c r="G48" s="1"/>
       <c r="H48" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I48" s="1"/>
     </row>

</xml_diff>

<commit_message>
[Excel & YAML] Fix Redundant Wording (Control 6.3 [EN])
</commit_message>
<xml_diff>
--- a/tools/excel/netherlands/cbw_nis2.xlsx
+++ b/tools/excel/netherlands/cbw_nis2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JulianDoloir\Desktop\Repos\intuitem\ciso-assistant-community\tools\excel\netherlands\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{782F7146-0AB4-4BA4-9DD2-943959E07E29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCBE50F9-E05F-4414-A49F-D916D97252F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2208" yWindow="504" windowWidth="19452" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
@@ -357,9 +357,6 @@
   </si>
   <si>
     <t>De entiteit heeft een volledige en actuele inventaris van haar leveranciers en dienstverleners en houdt deze bij. De entiteit houdt bij welke producten en diensten van leveranciers en dienstverleners worden afgenomen mede als de gemaakte afspreken over de afgenomen diensten en producten.</t>
-  </si>
-  <si>
-    <t>The entity has and maintains a complete and up-to-date inventory of its suppliers and service providers. The entity keeps track of which products and services are purchased from suppliers and service providers, also as well as the agreements made about the purchased services and products.</t>
   </si>
   <si>
     <t>Notre: For "description[en]", Control 6.3 was missing in OG Framework (probably because the English version wasn't up to date (v1.1 available only, while NL version was at v1.2)). NL has been translated to English for this control</t>
@@ -694,6 +691,9 @@
     <t>## Introduction
 The evaluation tool has been developed as a practical tool to support organizations in effectively gaining insight into their compliance with the Cybersecurity Act (Cbw) and the underlying Cybersecurity Decree (Cbb).
 The evaluation tool was developed to provide insight into the current state of cyber resilience and to identify potential for improvement, based on the requirements laid out in the Cbw and Cbb. The Cbw (NIS2) Control Framework does not replace current laws and regulations, but rather makes them transparent and manageable – see also the study report from p. 16 onwards. The Cbw and Cbb challenge organizations to implement the Cbw and Cbb through risk analysis and insight into their own organization. Employees of organizations are responsible for knowing and complying with the relevant laws and regulations. Furthermore, the specific context and characteristics of the organization and its environment should always be taken into account when using the tool.</t>
+  </si>
+  <si>
+    <t>The entity has and maintains a complete and up-to-date inventory of its suppliers and service providers. The entity keeps track of which products and services are purchased from suppliers and service providers, as well as the agreements made about the purchased services and products.</t>
   </si>
 </sst>
 </file>
@@ -1218,7 +1218,7 @@
         <v>21</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -1296,7 +1296,7 @@
         <v>21</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -1717,11 +1717,11 @@
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="3" t="s">
-        <v>89</v>
+        <v>179</v>
       </c>
       <c r="I19" s="1"/>
       <c r="J19" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
@@ -1731,12 +1731,12 @@
       </c>
       <c r="C20" s="1"/>
       <c r="D20" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
       <c r="G20" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
@@ -1749,21 +1749,21 @@
         <v>3</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D21" s="1"/>
       <c r="E21" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>95</v>
       </c>
       <c r="G21" s="1"/>
       <c r="H21" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I21" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
@@ -1774,16 +1774,16 @@
         <v>3</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I22" s="1"/>
     </row>
@@ -1795,16 +1795,16 @@
         <v>3</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I23" s="1"/>
     </row>
@@ -1815,12 +1815,12 @@
       </c>
       <c r="C24" s="1"/>
       <c r="D24" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
       <c r="G24" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
@@ -1833,16 +1833,16 @@
         <v>3</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
       <c r="H25" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="I25" s="1"/>
     </row>
@@ -1854,16 +1854,16 @@
         <v>3</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D26" s="1"/>
       <c r="E26" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
       <c r="H26" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I26" s="1"/>
     </row>
@@ -1874,12 +1874,12 @@
       </c>
       <c r="C27" s="1"/>
       <c r="D27" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
       <c r="G27" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
@@ -1892,21 +1892,21 @@
         <v>3</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D28" s="1"/>
       <c r="E28" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="F28" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>116</v>
       </c>
       <c r="G28" s="1"/>
       <c r="H28" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="I28" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
@@ -1916,12 +1916,12 @@
       </c>
       <c r="C29" s="1"/>
       <c r="D29" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
       <c r="G29" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
@@ -1934,16 +1934,16 @@
         <v>3</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D30" s="1"/>
       <c r="E30" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
       <c r="H30" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I30" s="1"/>
     </row>
@@ -1954,12 +1954,12 @@
       </c>
       <c r="C31" s="1"/>
       <c r="D31" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
       <c r="G31" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
@@ -1972,16 +1972,16 @@
         <v>3</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D32" s="1"/>
       <c r="E32" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
       <c r="H32" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I32" s="1"/>
     </row>
@@ -1992,12 +1992,12 @@
       </c>
       <c r="C33" s="1"/>
       <c r="D33" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
       <c r="G33" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
@@ -2010,21 +2010,21 @@
         <v>3</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D34" s="1"/>
       <c r="E34" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="F34" s="1" t="s">
         <v>132</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>133</v>
       </c>
       <c r="G34" s="1"/>
       <c r="H34" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="I34" s="1" t="s">
         <v>134</v>
-      </c>
-      <c r="I34" s="1" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
@@ -2035,16 +2035,16 @@
         <v>3</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D35" s="1"/>
       <c r="E35" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F35" s="1"/>
       <c r="G35" s="1"/>
       <c r="H35" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I35" s="1"/>
     </row>
@@ -2055,12 +2055,12 @@
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
       <c r="G36" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="H36" s="1"/>
       <c r="I36" s="1"/>
@@ -2073,21 +2073,21 @@
         <v>3</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D37" s="1"/>
       <c r="E37" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="F37" s="1" t="s">
         <v>142</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>143</v>
       </c>
       <c r="G37" s="1"/>
       <c r="H37" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="I37" s="1" t="s">
         <v>144</v>
-      </c>
-      <c r="I37" s="1" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
@@ -2097,12 +2097,12 @@
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
       <c r="G38" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
@@ -2114,12 +2114,12 @@
       </c>
       <c r="C39" s="1"/>
       <c r="D39" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
       <c r="G39" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H39" s="1"/>
       <c r="I39" s="1"/>
@@ -2132,21 +2132,21 @@
         <v>3</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D40" s="1"/>
       <c r="E40" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F40" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>152</v>
       </c>
       <c r="G40" s="1"/>
       <c r="H40" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="I40" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="I40" s="1" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="41" spans="1:9" ht="187.2" x14ac:dyDescent="0.3">
@@ -2157,21 +2157,21 @@
         <v>3</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D41" s="1"/>
       <c r="E41" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G41" s="1"/>
       <c r="H41" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
@@ -2181,12 +2181,12 @@
       </c>
       <c r="C42" s="1"/>
       <c r="D42" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
       <c r="G42" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H42" s="1"/>
       <c r="I42" s="1"/>
@@ -2198,12 +2198,12 @@
       </c>
       <c r="C43" s="1"/>
       <c r="D43" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
       <c r="G43" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H43" s="1"/>
       <c r="I43" s="1"/>
@@ -2216,21 +2216,21 @@
         <v>3</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D44" s="1"/>
       <c r="E44" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="F44" s="1" t="s">
         <v>163</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>164</v>
       </c>
       <c r="G44" s="1"/>
       <c r="H44" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="I44" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="I44" s="1" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.3">
@@ -2240,12 +2240,12 @@
       </c>
       <c r="C45" s="1"/>
       <c r="D45" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
       <c r="G45" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H45" s="1"/>
       <c r="I45" s="1"/>
@@ -2258,21 +2258,21 @@
         <v>3</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D46" s="1"/>
       <c r="E46" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="F46" s="1" t="s">
         <v>170</v>
-      </c>
-      <c r="F46" s="1" t="s">
-        <v>171</v>
       </c>
       <c r="G46" s="1"/>
       <c r="H46" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="I46" s="1" t="s">
         <v>172</v>
-      </c>
-      <c r="I46" s="1" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.3">
@@ -2282,12 +2282,12 @@
       </c>
       <c r="C47" s="1"/>
       <c r="D47" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
       <c r="G47" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H47" s="1"/>
       <c r="I47" s="1"/>
@@ -2300,16 +2300,16 @@
         <v>3</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D48" s="1"/>
       <c r="E48" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F48" s="1"/>
       <c r="G48" s="1"/>
       <c r="H48" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I48" s="1"/>
     </row>

</xml_diff>